<commit_message>
refactor(backend,frontend): broken, later be fixed
broken frontend, will be fixed later
</commit_message>
<xml_diff>
--- a/ExcelPreview/Assets/ExcelFile.xlsx
+++ b/ExcelPreview/Assets/ExcelFile.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\ExcelPreview\ExcelPreview\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6958471-46D9-4CAF-B5FD-E45983C4C790}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43D34B45-E028-4DC7-A3CC-0B51259FF827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3825" yWindow="0" windowWidth="14610" windowHeight="15480" xr2:uid="{D403B649-96F2-4878-B092-D7E2A2DF5859}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D403B649-96F2-4878-B092-D7E2A2DF5859}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -438,6 +439,7 @@
   <dimension ref="B3:E22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="3" max="3" width="18.28515625" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
@@ -629,4 +631,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{634625F4-B4F4-4D56-9F64-0CEBECDEA3DC}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(excelfile.xlsx): move chart to the sheet1
</commit_message>
<xml_diff>
--- a/ExcelPreview/Assets/ExcelFile.xlsx
+++ b/ExcelPreview/Assets/ExcelFile.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\ExcelPreview\ExcelPreview\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D67AE18-4E4F-4845-8FE6-A7AA43EC47F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38A7F997-F8C0-4323-9AF9-0F66077BC648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D403B649-96F2-4878-B092-D7E2A2DF5859}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="262" xr2:uid="{D403B649-96F2-4878-B092-D7E2A2DF5859}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$M$30</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1000,16 +1003,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>52387</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>238126</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>128587</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>142876</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1548,7 +1551,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>